<commit_message>
add e2e tests on local env
add e2e test cases

add testbooks

fix makefile

fix load workload env script

change workload kind to ddeployment

add test
</commit_message>
<xml_diff>
--- a/test-env/local/data/recommendations.xlsx
+++ b/test-env/local/data/recommendations.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30006"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11003"/>
   <workbookPr updateLinks="always"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\a470284\Mine\Projects\k8s-rightsizer\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mariano/Documents/projects/k8s-rightsizer/test-env/local/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B16DF485-9D8B-41FA-9602-9F4CAE924ED7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5CE3C533-B90D-1A44-9211-57C500878A48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-104" yWindow="-104" windowWidth="22326" windowHeight="11947" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="26200" windowHeight="15400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="HCO-Container Recommendatio DU" sheetId="3" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="41">
   <si>
     <t>Environment</t>
   </si>
@@ -51,9 +51,6 @@
     <t>Namespace</t>
   </si>
   <si>
-    <t>Type</t>
-  </si>
-  <si>
     <t>Workload Name</t>
   </si>
   <si>
@@ -87,16 +84,88 @@
     <t>MEM Limit Recommended [MB]</t>
   </si>
   <si>
-    <t>production</t>
-  </si>
-  <si>
-    <t>default</t>
-  </si>
-  <si>
-    <t>ReplicaSet</t>
-  </si>
-  <si>
-    <t>kubernetes-bootcamp</t>
+    <t>k8s-rightsizer-test</t>
+  </si>
+  <si>
+    <t>test-standard-rolling</t>
+  </si>
+  <si>
+    <t>Deployment</t>
+  </si>
+  <si>
+    <t>200m</t>
+  </si>
+  <si>
+    <t>128Mi</t>
+  </si>
+  <si>
+    <t>test-pdb-blocked</t>
+  </si>
+  <si>
+    <t>150m</t>
+  </si>
+  <si>
+    <t>256Mi</t>
+  </si>
+  <si>
+    <t>test-statefulset-ondelete</t>
+  </si>
+  <si>
+    <t>StatefulSet</t>
+  </si>
+  <si>
+    <t>300m</t>
+  </si>
+  <si>
+    <t>512Mi</t>
+  </si>
+  <si>
+    <t>test-degraded-app</t>
+  </si>
+  <si>
+    <t>100m</t>
+  </si>
+  <si>
+    <t>64Mi</t>
+  </si>
+  <si>
+    <t>test-fallback-oom</t>
+  </si>
+  <si>
+    <t>50m</t>
+  </si>
+  <si>
+    <t>5Mi</t>
+  </si>
+  <si>
+    <t>test-fallback-pending</t>
+  </si>
+  <si>
+    <t>8000m</t>
+  </si>
+  <si>
+    <t>16Gi</t>
+  </si>
+  <si>
+    <t>test-paused-workload</t>
+  </si>
+  <si>
+    <t>Kind</t>
+  </si>
+  <si>
+    <t>development</t>
+  </si>
+  <si>
+    <t>nginx</t>
+  </si>
+  <si>
+    <t>app-container</t>
+  </si>
+  <si>
+    <t>0Mi</t>
+  </si>
+  <si>
+    <t>0m</t>
   </si>
 </sst>
 </file>
@@ -141,18 +210,17 @@
       <family val="2"/>
     </font>
     <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF000FFB"/>
-      <name val="Calibri"/>
+      <sz val="10"/>
+      <color rgb="FF444746"/>
+      <name val="Google Sans Text"/>
       <family val="2"/>
     </font>
     <font>
-      <u/>
-      <sz val="11"/>
-      <color theme="1"/>
+      <sz val="12"/>
+      <color rgb="FF444746"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="4">
@@ -199,7 +267,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -208,17 +276,20 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="4">
-    <cellStyle name="Normale" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normale 2" xfId="1" xr:uid="{7C85B216-06C1-40AF-BF7C-757FD8850504}"/>
     <cellStyle name="Normale 2 2" xfId="3" xr:uid="{706D2D0A-9B96-4561-AACB-AC6A21B9F80E}"/>
     <cellStyle name="Normale 3" xfId="2" xr:uid="{D13E0992-DAA2-4C94-A1CC-D4E1D1A8FE45}"/>
@@ -520,116 +591,426 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{875B3D47-7E8A-4A9A-9CCE-2B38D6005361}">
-  <dimension ref="A1:N7"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.45"/>
+  <dimension ref="A1:N25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="21.5703125" style="5" customWidth="1"/>
-    <col min="2" max="2" width="42.28515625" style="5" customWidth="1"/>
-    <col min="3" max="3" width="29.28515625" style="5" customWidth="1"/>
-    <col min="4" max="4" width="28.42578125" style="5" customWidth="1"/>
-    <col min="5" max="5" width="28.140625" style="5" customWidth="1"/>
-    <col min="6" max="6" width="9.140625" style="5"/>
-    <col min="7" max="7" width="24" style="5" customWidth="1"/>
-    <col min="8" max="8" width="21.85546875" style="5" customWidth="1"/>
-    <col min="9" max="9" width="38" style="5" customWidth="1"/>
-    <col min="10" max="10" width="33.85546875" style="5" customWidth="1"/>
-    <col min="11" max="11" width="21" style="5" customWidth="1"/>
-    <col min="12" max="12" width="18.42578125" style="5" customWidth="1"/>
-    <col min="13" max="13" width="34.5703125" style="5" customWidth="1"/>
-    <col min="14" max="14" width="32.28515625" style="5" customWidth="1"/>
-    <col min="15" max="16384" width="9.140625" style="2"/>
+    <col min="1" max="1" width="21.5" style="4" customWidth="1"/>
+    <col min="2" max="2" width="42.33203125" style="4" customWidth="1"/>
+    <col min="3" max="3" width="29.33203125" style="4" customWidth="1"/>
+    <col min="4" max="4" width="28.5" style="4" customWidth="1"/>
+    <col min="5" max="5" width="28.1640625" style="4" customWidth="1"/>
+    <col min="6" max="6" width="9.1640625" style="4"/>
+    <col min="7" max="7" width="24" style="4" customWidth="1"/>
+    <col min="8" max="8" width="21.83203125" style="4" customWidth="1"/>
+    <col min="9" max="9" width="38" style="4" customWidth="1"/>
+    <col min="10" max="10" width="33.83203125" style="4" customWidth="1"/>
+    <col min="11" max="11" width="21" style="4" customWidth="1"/>
+    <col min="12" max="12" width="18.5" style="4" customWidth="1"/>
+    <col min="13" max="13" width="34.5" style="4" customWidth="1"/>
+    <col min="14" max="14" width="32.33203125" style="4" customWidth="1"/>
+    <col min="15" max="16384" width="9.1640625" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="8" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="K1" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="6" t="s">
+      <c r="L1" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="6" t="s">
+      <c r="M1" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="6" t="s">
+      <c r="N1" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="6" t="s">
+    </row>
+    <row r="2" spans="1:14" ht="16">
+      <c r="A2" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="B2" s="6" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="2" spans="1:14">
-      <c r="A2" s="3" t="s">
+      <c r="C2" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="D2" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="E2" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="F2" s="3">
+        <v>1</v>
+      </c>
+      <c r="G2" s="3"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="J2" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="K2" s="3"/>
+      <c r="L2" s="3"/>
+      <c r="M2" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="N2" s="3" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" ht="16">
+      <c r="A3" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="C3" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="D3" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="E3" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="F3" s="3">
+        <v>1</v>
+      </c>
+      <c r="G3" s="3"/>
+      <c r="H3" s="3"/>
+      <c r="I3" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="J3" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="K3" s="3"/>
+      <c r="L3" s="3"/>
+      <c r="M3" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="N3" s="3" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" ht="16">
+      <c r="A4" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="F4" s="3">
+        <v>1</v>
+      </c>
+      <c r="G4" s="3"/>
+      <c r="H4" s="3"/>
+      <c r="I4" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="J4" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="K4" s="3"/>
+      <c r="L4" s="3"/>
+      <c r="M4" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="N4" s="3" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" ht="16">
+      <c r="A5" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="F5" s="3">
+        <v>1</v>
+      </c>
+      <c r="G5" s="3"/>
+      <c r="H5" s="3"/>
+      <c r="I5" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="J5" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="K5" s="3"/>
+      <c r="L5" s="3"/>
+      <c r="M5" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="N5" s="3" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" ht="16">
+      <c r="A6" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="E6" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="F6" s="3">
+        <v>1</v>
+      </c>
+      <c r="G6" s="3"/>
+      <c r="H6" s="3"/>
+      <c r="I6" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="J6" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="K6" s="3"/>
+      <c r="L6" s="3"/>
+      <c r="M6" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="N6" s="3" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" ht="16">
+      <c r="A7" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="D7" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="E7" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="F7" s="3">
+        <v>1</v>
+      </c>
+      <c r="G7" s="3"/>
+      <c r="H7" s="3"/>
+      <c r="I7" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="J7" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="K7" s="3"/>
+      <c r="L7" s="3"/>
+      <c r="M7" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="N7" s="3" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" ht="16">
+      <c r="A8" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="E8" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="F8" s="3">
+        <v>1</v>
+      </c>
+      <c r="G8" s="3"/>
+      <c r="H8" s="3"/>
+      <c r="I8" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="J8" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="K8" s="3"/>
+      <c r="L8" s="3"/>
+      <c r="M8" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="E2" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="F2" s="3">
-        <v>2</v>
-      </c>
-      <c r="G2" s="3">
-        <v>200</v>
-      </c>
-      <c r="H2" s="3">
-        <v>200</v>
-      </c>
-      <c r="I2" s="3">
-        <v>50</v>
-      </c>
-      <c r="J2" s="3">
-        <v>50</v>
-      </c>
-      <c r="K2" s="3">
-        <v>256</v>
-      </c>
-      <c r="L2" s="3">
-        <v>256</v>
-      </c>
-      <c r="M2" s="3">
-        <v>10</v>
-      </c>
-      <c r="N2" s="3">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="7" spans="1:14">
-      <c r="A7" s="7"/>
+      <c r="N8" s="3" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14">
+      <c r="B12" s="6"/>
+      <c r="C12" s="6"/>
+      <c r="D12" s="6"/>
+      <c r="E12" s="6"/>
+      <c r="F12" s="6"/>
+    </row>
+    <row r="13" spans="1:14">
+      <c r="B13" s="6"/>
+      <c r="C13" s="6"/>
+      <c r="D13" s="6"/>
+      <c r="E13" s="6"/>
+      <c r="F13" s="6"/>
+    </row>
+    <row r="14" spans="1:14">
+      <c r="B14" s="6"/>
+      <c r="C14" s="6"/>
+      <c r="D14" s="6"/>
+      <c r="E14" s="6"/>
+      <c r="F14" s="6"/>
+    </row>
+    <row r="15" spans="1:14">
+      <c r="B15" s="6"/>
+      <c r="C15" s="6"/>
+      <c r="D15" s="6"/>
+      <c r="E15" s="6"/>
+      <c r="F15" s="6"/>
+    </row>
+    <row r="16" spans="1:14">
+      <c r="B16" s="6"/>
+      <c r="C16" s="6"/>
+      <c r="D16" s="6"/>
+      <c r="E16" s="6"/>
+      <c r="F16" s="6"/>
+    </row>
+    <row r="17" spans="2:7">
+      <c r="B17" s="6"/>
+      <c r="C17" s="6"/>
+      <c r="D17" s="6"/>
+      <c r="E17" s="6"/>
+      <c r="F17" s="6"/>
+    </row>
+    <row r="18" spans="2:7">
+      <c r="B18" s="6"/>
+      <c r="C18" s="6"/>
+      <c r="D18" s="6"/>
+      <c r="E18" s="6"/>
+      <c r="F18" s="6"/>
+    </row>
+    <row r="19" spans="2:7" ht="16">
+      <c r="B19" s="7"/>
+      <c r="C19" s="7"/>
+      <c r="D19" s="7"/>
+      <c r="E19" s="7"/>
+      <c r="F19" s="7"/>
+      <c r="G19" s="7"/>
+    </row>
+    <row r="20" spans="2:7" ht="16">
+      <c r="B20" s="7"/>
+      <c r="C20" s="7"/>
+      <c r="D20" s="7"/>
+      <c r="E20" s="7"/>
+      <c r="F20" s="7"/>
+      <c r="G20" s="7"/>
+    </row>
+    <row r="21" spans="2:7" ht="16">
+      <c r="B21" s="7"/>
+      <c r="C21" s="7"/>
+      <c r="D21" s="7"/>
+      <c r="E21" s="7"/>
+      <c r="F21" s="7"/>
+      <c r="G21" s="7"/>
+    </row>
+    <row r="22" spans="2:7" ht="16">
+      <c r="B22" s="7"/>
+      <c r="C22" s="7"/>
+      <c r="D22" s="7"/>
+      <c r="E22" s="7"/>
+      <c r="F22" s="7"/>
+      <c r="G22" s="7"/>
+    </row>
+    <row r="23" spans="2:7" ht="16">
+      <c r="B23" s="7"/>
+      <c r="C23" s="7"/>
+      <c r="D23" s="7"/>
+      <c r="E23" s="7"/>
+      <c r="F23" s="7"/>
+      <c r="G23" s="7"/>
+    </row>
+    <row r="24" spans="2:7" ht="16">
+      <c r="B24" s="7"/>
+      <c r="C24" s="7"/>
+      <c r="D24" s="7"/>
+      <c r="E24" s="7"/>
+      <c r="F24" s="7"/>
+      <c r="G24" s="7"/>
+    </row>
+    <row r="25" spans="2:7" ht="16">
+      <c r="B25" s="7"/>
+      <c r="C25" s="7"/>
+      <c r="D25" s="7"/>
+      <c r="E25" s="7"/>
+      <c r="F25" s="7"/>
+      <c r="G25" s="7"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:N2" xr:uid="{875B3D47-7E8A-4A9A-9CCE-2B38D6005361}"/>
@@ -642,15 +1023,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100A9D9B79EAD5BA94E9A3F379047946D7F" ma:contentTypeVersion="6" ma:contentTypeDescription="Creare un nuovo documento." ma:contentTypeScope="" ma:versionID="7e4e56769a6e72cb5ab09fe359caccfe">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="e9d8133e-f311-40cb-b671-5c6149caa565" xmlns:ns3="8762e784-f5b5-458b-8d6e-f5b044ec62de" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="36c6d8eefc5e52647de0e841ad48104e" ns2:_="" ns3:_="">
     <xsd:import namespace="e9d8133e-f311-40cb-b671-5c6149caa565"/>
@@ -827,6 +1199,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement/>
@@ -834,13 +1215,37 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C0BB01DB-2273-48CA-9212-17EA76FB34AA}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1FB5485A-4DB0-46AA-854B-F0993EB63B4F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="e9d8133e-f311-40cb-b671-5c6149caa565"/>
+    <ds:schemaRef ds:uri="8762e784-f5b5-458b-8d6e-f5b044ec62de"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1FB5485A-4DB0-46AA-854B-F0993EB63B4F}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C0BB01DB-2273-48CA-9212-17EA76FB34AA}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AA8BD82F-AA6D-48FD-8510-6ED9BD04899D}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AA8BD82F-AA6D-48FD-8510-6ED9BD04899D}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>